<commit_message>
Create core and kw
</commit_message>
<xml_diff>
--- a/framework/data/excel/cart_hybrid.xlsx
+++ b/framework/data/excel/cart_hybrid.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DA4\DA4_hybrid_selenium_framework\framework\data\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E50A79D3-0FD5-47DB-BC42-CFA8ED778A78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{347E2CC4-6C05-4734-A909-EE24AC5CD66A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="test_step" sheetId="1" r:id="rId1"/>
@@ -514,7 +514,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -534,6 +534,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE9EFF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -564,7 +576,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -587,6 +599,20 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2251,83 +2277,83 @@
         <v>134</v>
       </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
+    <row r="10" spans="1:24" s="10" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="8" t="s">
         <v>147</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2">
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8">
         <v>-1</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="J10" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="K10" s="2" t="s">
+      <c r="K10" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="L10" s="2" t="s">
+      <c r="L10" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="M10" s="2"/>
-      <c r="N10" s="2"/>
-      <c r="O10" s="2"/>
-      <c r="P10" s="2"/>
-      <c r="Q10" s="2"/>
-      <c r="R10" s="2"/>
-      <c r="S10" s="2"/>
-      <c r="T10" s="2"/>
-      <c r="U10" s="2"/>
-      <c r="V10" s="2"/>
-      <c r="W10" s="2"/>
-      <c r="X10" s="7" t="s">
+      <c r="M10" s="8"/>
+      <c r="N10" s="8"/>
+      <c r="O10" s="8"/>
+      <c r="P10" s="8"/>
+      <c r="Q10" s="8"/>
+      <c r="R10" s="8"/>
+      <c r="S10" s="8"/>
+      <c r="T10" s="8"/>
+      <c r="U10" s="8"/>
+      <c r="V10" s="8"/>
+      <c r="W10" s="8"/>
+      <c r="X10" s="9" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
+    <row r="11" spans="1:24" s="13" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="11" t="s">
         <v>148</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4" t="s">
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
+      <c r="I11" s="11" t="s">
         <v>138</v>
       </c>
-      <c r="J11" s="4" t="s">
+      <c r="J11" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="K11" s="4" t="s">
+      <c r="K11" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="L11" s="4" t="s">
+      <c r="L11" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="M11" s="4"/>
-      <c r="N11" s="4"/>
-      <c r="O11" s="4"/>
-      <c r="P11" s="4"/>
-      <c r="Q11" s="4"/>
-      <c r="R11" s="4"/>
-      <c r="S11" s="4"/>
-      <c r="T11" s="4"/>
-      <c r="U11" s="4"/>
-      <c r="V11" s="4"/>
-      <c r="W11" s="4"/>
-      <c r="X11" s="6" t="s">
+      <c r="M11" s="11"/>
+      <c r="N11" s="11"/>
+      <c r="O11" s="11"/>
+      <c r="P11" s="11"/>
+      <c r="Q11" s="11"/>
+      <c r="R11" s="11"/>
+      <c r="S11" s="11"/>
+      <c r="T11" s="11"/>
+      <c r="U11" s="11"/>
+      <c r="V11" s="11"/>
+      <c r="W11" s="11"/>
+      <c r="X11" s="12" t="s">
         <v>139</v>
       </c>
     </row>

</xml_diff>